<commit_message>
crawling to a finished template - not there yet
</commit_message>
<xml_diff>
--- a/metadata/MIAFPE/MIAFPE_template_v1.1.xlsx
+++ b/metadata/MIAFPE/MIAFPE_template_v1.1.xlsx
@@ -18,6 +18,15 @@
     <sheet name="ExperimentalDesign" sheetId="8" state="visible" r:id="rId10"/>
     <sheet name="Observation" sheetId="9" state="visible" r:id="rId11"/>
     <sheet name="ObservationUnit" sheetId="10" state="visible" r:id="rId12"/>
+    <sheet name="System" sheetId="11" state="visible" r:id="rId13"/>
+    <sheet name="Platform" sheetId="12" state="visible" r:id="rId14"/>
+    <sheet name="Sensor" sheetId="13" state="visible" r:id="rId15"/>
+    <sheet name="ObservedVariable" sheetId="14" state="visible" r:id="rId16"/>
+    <sheet name="Factor" sheetId="15" state="visible" r:id="rId17"/>
+    <sheet name="Sample" sheetId="16" state="visible" r:id="rId18"/>
+    <sheet name="BiologicalMaterial" sheetId="17" state="visible" r:id="rId19"/>
+    <sheet name="Event" sheetId="18" state="visible" r:id="rId20"/>
+    <sheet name="Environment" sheetId="19" state="visible" r:id="rId21"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -29,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="775" uniqueCount="359">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="817" uniqueCount="401">
   <si>
     <t xml:space="preserve">Sheet Name</t>
   </si>
@@ -856,6 +865,9 @@
     <t xml:space="preserve">Spatial Distribution</t>
   </si>
   <si>
+    <t xml:space="preserve">Type and value of a spatial coordinate (georeference or relative) or level of observation (plot 45, subblock 7, block 2) provided as a key-value pair of the form type:value. Levels of observation must be consistent with those listed in the Study section.</t>
+  </si>
+  <si>
     <t xml:space="preserve">hasSpatialDistribution</t>
   </si>
   <si>
@@ -865,6 +877,9 @@
     <t xml:space="preserve">Spatial Distribution Type</t>
   </si>
   <si>
+    <t xml:space="preserve">Type of Spatial Detribution.</t>
+  </si>
+  <si>
     <t xml:space="preserve">hasSpatialDistributionType</t>
   </si>
   <si>
@@ -880,6 +895,9 @@
     <t xml:space="preserve">Experimental Factor</t>
   </si>
   <si>
+    <t xml:space="preserve">List of Experimental Factor Identifier (semi-colon separated) </t>
+  </si>
+  <si>
     <t xml:space="preserve">Observed Variable</t>
   </si>
   <si>
@@ -898,16 +916,133 @@
     <t xml:space="preserve">Variable Name</t>
   </si>
   <si>
+    <t xml:space="preserve">Name of the Variable.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anthesis computed in growing degree days</t>
+  </si>
+  <si>
     <t xml:space="preserve">Variable Accession Number</t>
   </si>
   <si>
+    <t xml:space="preserve">URI of an Ontology Term (for example Crop Ontology).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CO_322:0000794</t>
+  </si>
+  <si>
     <t xml:space="preserve">Trait</t>
   </si>
   <si>
+    <t xml:space="preserve">Name of the (plant or environmental) trait under observation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anthesis time;  Reproductive growth time</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trait Entity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entity (part of the plant, whole plant, group of plant e.g. canopy) on which the trait has been measured</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Leaf</t>
+  </si>
+  <si>
     <t xml:space="preserve">Trait Entity Accession Number</t>
   </si>
   <si>
+    <t xml:space="preserve">Accession number of the trait entity in a suitable controlled vocabulary (Plant Ontology).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">http://purl.obolibrary.org/obo/PO_0025034</t>
+  </si>
+  <si>
     <t xml:space="preserve">Trait Characteristics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Characteristic measured. It can be a morphological characteristic (size, volume, surface), a molecular characteristic (sugar concentration), etc...</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Area</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trait Characteristic Accession number</t>
+  </si>
+  <si>
+    <t xml:space="preserve">http://purl.obolibrary.org/obo/PATO_0001323</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trait accession number</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Accession number of the trait in a suitable controlled vocabulary (Crop Ontology, Trait Ontology).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CO_322:0000030; TO:0000366</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Method</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Name of the method of observation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Growing degree days to anthesis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Method accession number</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Accession number of the method in a suitable controlled vocabulary (Crop Ontology, Trait Ontology).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CO_322:0000189</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Method description</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Textual description of the method, which may extend a method defined in an external reference with specific parameters, e.g. growth stage, inoculation precise organ (leaf number)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Days to anthesis for male flowering was measured in thermal time (GDD: growing degree-days) according to Ritchie J, NeSmith D (1991;Temperature and crop development. Modeling plant and soil systems American Society of Agronomy Madison, Wisconsin USA) with TBASE=8°C and T0=30°C. ; Plant height was measured at 5 years with a ruler, one year after Botritis inoculation.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reference associated to the method</t>
+  </si>
+  <si>
+    <t xml:space="preserve">URI/DOI of reference describing the method.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://doi.org/10.2134/agronmonogr31.c2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scale</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Name of the scale associated with the variable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">°C day</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scale accession number</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Accession number of the scale in a suitable controlled vocabulary (Crop Ontology).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CO_322:0000510</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Time scale</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Name of the scale or unit of time with which observations of this type were recorded in the data file (for time series studies).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Growing degree day (GDD); Date/Time</t>
   </si>
   <si>
     <t xml:space="preserve">The object of a study is to ascertain the impact of one or more factors on the biological material. Thus, a factor is, by definition a condition that varies between observation units, which may be biotic (pest, disease interaction) or abiotic (treatment and cultural practice) in nature. Depending on the level of the data, an experimental factor can be either  "what is the factor applied to the plant" (i.e. Unwatered), or the "environmental characterisation" (i.e. if no rain on unwatered plant : Drought ;  if rain on unwatered plant: Irrigated) </t>
@@ -1112,10 +1247,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="General"/>
-    <numFmt numFmtId="166" formatCode="yyyy\-mm\-dd"/>
+    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
   <fonts count="12">
     <font>
@@ -1161,11 +1295,6 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
       <b val="true"/>
       <sz val="10"/>
       <name val="Arial"/>
@@ -1194,6 +1323,11 @@
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="7">
@@ -1317,7 +1451,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="46">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1378,10 +1512,6 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1390,7 +1520,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1398,7 +1528,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1418,11 +1548,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1434,7 +1564,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1450,7 +1580,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1458,7 +1588,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1486,15 +1624,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1681,7 +1819,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M181"/>
+  <dimension ref="A1:M189"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="21.21"/>
@@ -1698,7 +1836,7 @@
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="13" style="1" width="11.53"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="30.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1736,7 +1874,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="47.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
         <v>12</v>
       </c>
@@ -1768,7 +1906,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="36.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7"/>
       <c r="B3" s="8" t="s">
         <v>17</v>
@@ -1804,7 +1942,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="59.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7"/>
       <c r="B4" s="11" t="s">
         <v>23</v>
@@ -1840,7 +1978,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="105.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7"/>
       <c r="B5" s="11" t="s">
         <v>29</v>
@@ -1876,7 +2014,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="47.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7"/>
       <c r="B6" s="11" t="s">
         <v>35</v>
@@ -1912,7 +2050,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="47.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7"/>
       <c r="B7" s="11" t="s">
         <v>40</v>
@@ -1948,7 +2086,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="36.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7"/>
       <c r="B8" s="11" t="s">
         <v>44</v>
@@ -1984,7 +2122,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="34.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7"/>
       <c r="B9" s="14" t="s">
         <v>49</v>
@@ -2043,7 +2181,7 @@
       </c>
       <c r="K10" s="12"/>
     </row>
-    <row r="11" customFormat="false" ht="47.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7"/>
       <c r="B11" s="14" t="s">
         <v>57</v>
@@ -2051,7 +2189,7 @@
       <c r="C11" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="D11" s="15" t="s">
+      <c r="D11" s="10" t="s">
         <v>59</v>
       </c>
       <c r="E11" s="1" t="s">
@@ -2081,71 +2219,71 @@
     </row>
     <row r="12" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7"/>
-      <c r="B12" s="16" t="s">
+      <c r="B12" s="15" t="s">
         <v>63</v>
       </c>
-      <c r="C12" s="17" t="s">
+      <c r="C12" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="D12" s="17"/>
-      <c r="E12" s="18" t="s">
+      <c r="D12" s="16"/>
+      <c r="E12" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="F12" s="17" t="s">
+      <c r="F12" s="16" t="s">
         <v>66</v>
       </c>
-      <c r="G12" s="19" t="s">
+      <c r="G12" s="18" t="s">
         <v>67</v>
       </c>
-      <c r="H12" s="17" t="s">
-        <v>15</v>
-      </c>
-      <c r="I12" s="17" t="str">
+      <c r="H12" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="I12" s="16" t="str">
         <f aca="false">_xlfn.CONCAT(H12, G12)</f>
         <v>http://purl.org/ppeo/ppeo.owl#hasDataFile</v>
       </c>
-      <c r="J12" s="20" t="str">
+      <c r="J12" s="19" t="str">
         <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G12)</f>
         <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#hasDataFile</v>
       </c>
-      <c r="K12" s="20"/>
-    </row>
-    <row r="13" customFormat="false" ht="36.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="21" t="s">
+      <c r="K12" s="19"/>
+    </row>
+    <row r="13" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B13" s="22"/>
-      <c r="C13" s="23" t="s">
+      <c r="B13" s="21"/>
+      <c r="C13" s="22" t="s">
         <v>69</v>
       </c>
-      <c r="D13" s="23"/>
-      <c r="E13" s="22"/>
-      <c r="F13" s="22" t="s">
+      <c r="D13" s="22"/>
+      <c r="E13" s="21"/>
+      <c r="F13" s="21" t="s">
         <v>70</v>
       </c>
-      <c r="G13" s="22" t="s">
+      <c r="G13" s="21" t="s">
         <v>68</v>
       </c>
-      <c r="H13" s="23" t="s">
-        <v>15</v>
-      </c>
-      <c r="I13" s="23" t="str">
+      <c r="H13" s="22" t="s">
+        <v>15</v>
+      </c>
+      <c r="I13" s="22" t="str">
         <f aca="false">_xlfn.CONCAT(H13, LOWER(G13))</f>
         <v>http://purl.org/ppeo/ppeo.owl#study</v>
       </c>
-      <c r="J13" s="22" t="str">
+      <c r="J13" s="21" t="str">
         <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G13)</f>
         <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#Study</v>
       </c>
-      <c r="K13" s="23" t="s">
+      <c r="K13" s="22" t="s">
         <v>71</v>
       </c>
-      <c r="L13" s="23" t="s">
+      <c r="L13" s="22" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="24"/>
+      <c r="A14" s="23"/>
       <c r="B14" s="8" t="s">
         <v>73</v>
       </c>
@@ -2181,7 +2319,7 @@
       </c>
     </row>
     <row r="15" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="24"/>
+      <c r="A15" s="23"/>
       <c r="B15" s="11" t="s">
         <v>77</v>
       </c>
@@ -2214,7 +2352,7 @@
       </c>
     </row>
     <row r="16" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="24"/>
+      <c r="A16" s="23"/>
       <c r="B16" s="11" t="s">
         <v>80</v>
       </c>
@@ -2247,7 +2385,7 @@
       </c>
     </row>
     <row r="17" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="24"/>
+      <c r="A17" s="23"/>
       <c r="B17" s="11" t="s">
         <v>83</v>
       </c>
@@ -2277,7 +2415,7 @@
       <c r="K17" s="12"/>
     </row>
     <row r="18" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="24"/>
+      <c r="A18" s="23"/>
       <c r="B18" s="11" t="s">
         <v>86</v>
       </c>
@@ -2307,14 +2445,14 @@
       <c r="K18" s="12"/>
     </row>
     <row r="19" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="24"/>
+      <c r="A19" s="23"/>
       <c r="B19" s="11" t="s">
         <v>89</v>
       </c>
       <c r="C19" s="10" t="s">
         <v>90</v>
       </c>
-      <c r="E19" s="25" t="s">
+      <c r="E19" s="24" t="s">
         <v>91</v>
       </c>
       <c r="F19" s="1" t="s">
@@ -2337,14 +2475,14 @@
       <c r="K19" s="12"/>
     </row>
     <row r="20" customFormat="false" ht="34.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="24"/>
+      <c r="A20" s="23"/>
       <c r="B20" s="14" t="s">
         <v>93</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="E20" s="25" t="s">
+      <c r="E20" s="24" t="s">
         <v>93</v>
       </c>
       <c r="F20" s="1" t="s">
@@ -2367,14 +2505,14 @@
       <c r="K20" s="12"/>
     </row>
     <row r="21" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="24"/>
+      <c r="A21" s="23"/>
       <c r="B21" s="14" t="s">
         <v>96</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="E21" s="25" t="s">
+      <c r="E21" s="24" t="s">
         <v>98</v>
       </c>
       <c r="F21" s="1" t="s">
@@ -2397,38 +2535,38 @@
       <c r="K21" s="12"/>
     </row>
     <row r="22" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="24"/>
-      <c r="B22" s="16" t="s">
+      <c r="A22" s="23"/>
+      <c r="B22" s="15" t="s">
         <v>100</v>
       </c>
-      <c r="C22" s="17" t="s">
+      <c r="C22" s="16" t="s">
         <v>101</v>
       </c>
-      <c r="D22" s="17"/>
-      <c r="E22" s="18" t="s">
+      <c r="D22" s="16"/>
+      <c r="E22" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="F22" s="17" t="s">
+      <c r="F22" s="16" t="s">
         <v>66</v>
       </c>
-      <c r="G22" s="19" t="s">
+      <c r="G22" s="18" t="s">
         <v>67</v>
       </c>
-      <c r="H22" s="17" t="s">
-        <v>15</v>
-      </c>
-      <c r="I22" s="17" t="str">
+      <c r="H22" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="I22" s="16" t="str">
         <f aca="false">_xlfn.CONCAT(H22, G22)</f>
         <v>http://purl.org/ppeo/ppeo.owl#hasDataFile</v>
       </c>
-      <c r="J22" s="20" t="str">
+      <c r="J22" s="19" t="str">
         <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G22)</f>
         <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#hasDataFile</v>
       </c>
-      <c r="K22" s="20"/>
-    </row>
-    <row r="23" customFormat="false" ht="36.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="26" t="s">
+      <c r="K22" s="19"/>
+    </row>
+    <row r="23" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="25" t="s">
         <v>93</v>
       </c>
       <c r="B23" s="4"/>
@@ -2520,34 +2658,34 @@
     </row>
     <row r="26" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="7"/>
-      <c r="B26" s="27" t="s">
+      <c r="B26" s="26" t="s">
         <v>107</v>
       </c>
-      <c r="C26" s="28" t="s">
+      <c r="C26" s="27" t="s">
         <v>108</v>
       </c>
-      <c r="D26" s="28"/>
-      <c r="E26" s="29" t="s">
+      <c r="D26" s="27"/>
+      <c r="E26" s="28" t="s">
         <v>26</v>
       </c>
-      <c r="F26" s="28" t="s">
+      <c r="F26" s="27" t="s">
         <v>70</v>
       </c>
-      <c r="G26" s="28" t="s">
+      <c r="G26" s="27" t="s">
         <v>27</v>
       </c>
-      <c r="H26" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="I26" s="28" t="str">
+      <c r="H26" s="27" t="s">
+        <v>15</v>
+      </c>
+      <c r="I26" s="27" t="str">
         <f aca="false">_xlfn.CONCAT(H26, G26)</f>
         <v>http://purl.org/ppeo/ppeo.owl#hasName</v>
       </c>
-      <c r="J26" s="28" t="str">
+      <c r="J26" s="27" t="str">
         <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G26)</f>
         <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#hasName</v>
       </c>
-      <c r="K26" s="30"/>
+      <c r="K26" s="29"/>
       <c r="L26" s="1" t="s">
         <v>109</v>
       </c>
@@ -2557,34 +2695,34 @@
     </row>
     <row r="27" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="7"/>
-      <c r="B27" s="27" t="s">
+      <c r="B27" s="26" t="s">
         <v>111</v>
       </c>
-      <c r="C27" s="28" t="s">
+      <c r="C27" s="27" t="s">
         <v>112</v>
       </c>
-      <c r="D27" s="28"/>
-      <c r="E27" s="28" t="s">
+      <c r="D27" s="27"/>
+      <c r="E27" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="F27" s="28" t="s">
+      <c r="F27" s="27" t="s">
         <v>70</v>
       </c>
-      <c r="G27" s="28" t="s">
+      <c r="G27" s="27" t="s">
         <v>113</v>
       </c>
-      <c r="H27" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="I27" s="28" t="str">
+      <c r="H27" s="27" t="s">
+        <v>15</v>
+      </c>
+      <c r="I27" s="27" t="str">
         <f aca="false">_xlfn.CONCAT(H27, G27)</f>
         <v>http://purl.org/ppeo/ppeo.owl#hasCountryCode</v>
       </c>
-      <c r="J27" s="28" t="str">
+      <c r="J27" s="27" t="str">
         <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G27)</f>
         <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#hasCountryCode</v>
       </c>
-      <c r="K27" s="30"/>
+      <c r="K27" s="29"/>
     </row>
     <row r="28" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="7"/>
@@ -2684,34 +2822,34 @@
     </row>
     <row r="31" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="7"/>
-      <c r="B31" s="27" t="s">
+      <c r="B31" s="26" t="s">
         <v>127</v>
       </c>
-      <c r="C31" s="28" t="s">
+      <c r="C31" s="27" t="s">
         <v>128</v>
       </c>
-      <c r="D31" s="28"/>
-      <c r="E31" s="28" t="s">
+      <c r="D31" s="27"/>
+      <c r="E31" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="F31" s="28" t="s">
+      <c r="F31" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="G31" s="28" t="s">
+      <c r="G31" s="27" t="s">
         <v>33</v>
       </c>
-      <c r="H31" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="I31" s="28" t="str">
+      <c r="H31" s="27" t="s">
+        <v>15</v>
+      </c>
+      <c r="I31" s="27" t="str">
         <f aca="false">_xlfn.CONCAT(H31,G31)</f>
         <v>http://purl.org/ppeo/ppeo.owl#hasDescription</v>
       </c>
-      <c r="J31" s="28" t="str">
+      <c r="J31" s="27" t="str">
         <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G31)</f>
         <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#hasDescription</v>
       </c>
-      <c r="K31" s="28" t="s">
+      <c r="K31" s="27" t="s">
         <v>129</v>
       </c>
       <c r="L31" s="1" t="s">
@@ -2721,36 +2859,36 @@
         <v>131</v>
       </c>
     </row>
-    <row r="32" s="31" customFormat="true" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" s="30" customFormat="true" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="7"/>
-      <c r="B32" s="27" t="s">
+      <c r="B32" s="26" t="s">
         <v>132</v>
       </c>
-      <c r="C32" s="28" t="s">
+      <c r="C32" s="27" t="s">
         <v>133</v>
       </c>
-      <c r="D32" s="28"/>
-      <c r="E32" s="28" t="s">
+      <c r="D32" s="27"/>
+      <c r="E32" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="F32" s="28" t="s">
+      <c r="F32" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="G32" s="28" t="s">
+      <c r="G32" s="27" t="s">
         <v>134</v>
       </c>
-      <c r="H32" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="I32" s="28" t="str">
+      <c r="H32" s="27" t="s">
+        <v>15</v>
+      </c>
+      <c r="I32" s="27" t="str">
         <f aca="false">_xlfn.CONCAT(H32,G32)</f>
         <v>http://purl.org/ppeo/ppeo.owl#hasGrowthFacilityType</v>
       </c>
-      <c r="J32" s="28" t="str">
+      <c r="J32" s="27" t="str">
         <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G32)</f>
         <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#hasGrowthFacilityType</v>
       </c>
-      <c r="K32" s="28" t="s">
+      <c r="K32" s="27" t="s">
         <v>129</v>
       </c>
       <c r="L32" s="1"/>
@@ -2758,95 +2896,95 @@
     </row>
     <row r="33" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="7"/>
-      <c r="B33" s="27" t="s">
+      <c r="B33" s="26" t="s">
         <v>135</v>
       </c>
-      <c r="C33" s="28" t="s">
+      <c r="C33" s="27" t="s">
         <v>136</v>
       </c>
-      <c r="D33" s="28"/>
-      <c r="E33" s="28" t="s">
+      <c r="D33" s="27"/>
+      <c r="E33" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="F33" s="28" t="s">
+      <c r="F33" s="27" t="s">
         <v>32</v>
       </c>
-      <c r="G33" s="28" t="s">
+      <c r="G33" s="27" t="s">
         <v>137</v>
       </c>
-      <c r="H33" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="I33" s="28" t="str">
+      <c r="H33" s="27" t="s">
+        <v>15</v>
+      </c>
+      <c r="I33" s="27" t="str">
         <f aca="false">_xlfn.CONCAT(H33,G33)</f>
         <v>http://purl.org/ppeo/ppeo.owl#hasExternalIdentifier</v>
       </c>
-      <c r="J33" s="28" t="str">
+      <c r="J33" s="27" t="str">
         <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G33)</f>
         <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#hasExternalIdentifier</v>
       </c>
-      <c r="K33" s="28"/>
+      <c r="K33" s="27"/>
     </row>
     <row r="34" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="7"/>
-      <c r="B34" s="32" t="s">
+      <c r="B34" s="31" t="s">
         <v>138</v>
       </c>
-      <c r="C34" s="20" t="s">
+      <c r="C34" s="19" t="s">
         <v>139</v>
       </c>
-      <c r="D34" s="20"/>
-      <c r="E34" s="18" t="s">
+      <c r="D34" s="19"/>
+      <c r="E34" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="F34" s="20" t="s">
+      <c r="F34" s="19" t="s">
         <v>66</v>
       </c>
-      <c r="G34" s="20" t="s">
+      <c r="G34" s="19" t="s">
         <v>67</v>
       </c>
-      <c r="H34" s="17" t="s">
-        <v>15</v>
-      </c>
-      <c r="I34" s="17" t="str">
+      <c r="H34" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="I34" s="16" t="str">
         <f aca="false">_xlfn.CONCAT(H34, G34)</f>
         <v>http://purl.org/ppeo/ppeo.owl#hasDataFile</v>
       </c>
-      <c r="J34" s="20" t="str">
+      <c r="J34" s="19" t="str">
         <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G34)</f>
         <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#hasDataFile</v>
       </c>
-      <c r="K34" s="20"/>
+      <c r="K34" s="19"/>
     </row>
     <row r="35" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="33" t="s">
+      <c r="A35" s="32" t="s">
         <v>91</v>
       </c>
-      <c r="B35" s="22"/>
-      <c r="C35" s="23" t="s">
+      <c r="B35" s="21"/>
+      <c r="C35" s="22" t="s">
         <v>140</v>
       </c>
-      <c r="D35" s="23"/>
-      <c r="E35" s="22"/>
-      <c r="F35" s="22"/>
-      <c r="G35" s="22" t="s">
+      <c r="D35" s="22"/>
+      <c r="E35" s="21"/>
+      <c r="F35" s="21"/>
+      <c r="G35" s="21" t="s">
         <v>91</v>
       </c>
-      <c r="H35" s="23" t="s">
-        <v>15</v>
-      </c>
-      <c r="I35" s="23" t="str">
+      <c r="H35" s="22" t="s">
+        <v>15</v>
+      </c>
+      <c r="I35" s="22" t="str">
         <f aca="false">_xlfn.CONCAT(H35, LOWER(G35))</f>
         <v>http://purl.org/ppeo/ppeo.owl#institution</v>
       </c>
-      <c r="J35" s="22" t="str">
+      <c r="J35" s="21" t="str">
         <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G35)</f>
         <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#Institution</v>
       </c>
-      <c r="K35" s="22"/>
+      <c r="K35" s="21"/>
     </row>
     <row r="36" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="24"/>
+      <c r="A36" s="23"/>
       <c r="B36" s="11" t="s">
         <v>20</v>
       </c>
@@ -2878,7 +3016,7 @@
       </c>
     </row>
     <row r="37" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="24"/>
+      <c r="A37" s="23"/>
       <c r="B37" s="11" t="s">
         <v>142</v>
       </c>
@@ -2907,7 +3045,7 @@
       </c>
     </row>
     <row r="38" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="24"/>
+      <c r="A38" s="23"/>
       <c r="B38" s="11" t="s">
         <v>144</v>
       </c>
@@ -2936,72 +3074,72 @@
       </c>
     </row>
     <row r="39" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="24"/>
-      <c r="B39" s="27" t="s">
+      <c r="A39" s="23"/>
+      <c r="B39" s="26" t="s">
         <v>107</v>
       </c>
-      <c r="C39" s="28" t="s">
+      <c r="C39" s="27" t="s">
         <v>108</v>
       </c>
-      <c r="D39" s="28"/>
-      <c r="E39" s="28" t="s">
+      <c r="D39" s="27"/>
+      <c r="E39" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="F39" s="28" t="s">
+      <c r="F39" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="G39" s="28" t="s">
+      <c r="G39" s="27" t="s">
         <v>27</v>
       </c>
-      <c r="H39" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="I39" s="28" t="str">
+      <c r="H39" s="27" t="s">
+        <v>15</v>
+      </c>
+      <c r="I39" s="27" t="str">
         <f aca="false">_xlfn.CONCAT(H39,G39)</f>
         <v>http://purl.org/ppeo/ppeo.owl#hasName</v>
       </c>
-      <c r="J39" s="28" t="str">
+      <c r="J39" s="27" t="str">
         <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G39)</f>
         <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#hasName</v>
       </c>
-      <c r="K39" s="28"/>
+      <c r="K39" s="27"/>
       <c r="L39" s="1" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="24"/>
-      <c r="B40" s="27" t="s">
+      <c r="A40" s="23"/>
+      <c r="B40" s="26" t="s">
         <v>111</v>
       </c>
-      <c r="C40" s="28" t="s">
+      <c r="C40" s="27" t="s">
         <v>112</v>
       </c>
-      <c r="D40" s="28"/>
-      <c r="E40" s="28" t="s">
+      <c r="D40" s="27"/>
+      <c r="E40" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="F40" s="28" t="s">
+      <c r="F40" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="G40" s="28" t="s">
+      <c r="G40" s="27" t="s">
         <v>113</v>
       </c>
-      <c r="H40" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="I40" s="28" t="str">
+      <c r="H40" s="27" t="s">
+        <v>15</v>
+      </c>
+      <c r="I40" s="27" t="str">
         <f aca="false">_xlfn.CONCAT(H40,G40)</f>
         <v>http://purl.org/ppeo/ppeo.owl#hasCountryCode</v>
       </c>
-      <c r="J40" s="28" t="str">
+      <c r="J40" s="27" t="str">
         <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G40)</f>
         <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#hasCountryCode</v>
       </c>
-      <c r="K40" s="28"/>
+      <c r="K40" s="27"/>
     </row>
     <row r="41" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="24"/>
+      <c r="A41" s="23"/>
       <c r="B41" s="11" t="s">
         <v>147</v>
       </c>
@@ -3030,7 +3168,7 @@
       </c>
     </row>
     <row r="42" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="24"/>
+      <c r="A42" s="23"/>
       <c r="B42" s="11" t="s">
         <v>150</v>
       </c>
@@ -3052,7 +3190,7 @@
       </c>
     </row>
     <row r="43" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="24"/>
+      <c r="A43" s="23"/>
       <c r="B43" s="11" t="s">
         <v>152</v>
       </c>
@@ -3074,7 +3212,7 @@
       </c>
     </row>
     <row r="44" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="24"/>
+      <c r="A44" s="23"/>
       <c r="B44" s="11" t="s">
         <v>154</v>
       </c>
@@ -3096,7 +3234,7 @@
       </c>
     </row>
     <row r="45" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="24"/>
+      <c r="A45" s="23"/>
       <c r="B45" s="11" t="s">
         <v>156</v>
       </c>
@@ -3118,7 +3256,7 @@
       </c>
     </row>
     <row r="46" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="24"/>
+      <c r="A46" s="23"/>
       <c r="B46" s="11" t="s">
         <v>158</v>
       </c>
@@ -3140,7 +3278,7 @@
       </c>
     </row>
     <row r="47" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="24"/>
+      <c r="A47" s="23"/>
       <c r="B47" s="11" t="s">
         <v>160</v>
       </c>
@@ -3168,8 +3306,8 @@
         <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#hasExternalIdentifier</v>
       </c>
     </row>
-    <row r="48" s="31" customFormat="true" ht="45.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="26" t="s">
+    <row r="48" s="30" customFormat="true" ht="45.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="25" t="s">
         <v>96</v>
       </c>
       <c r="B48" s="4"/>
@@ -3261,7 +3399,7 @@
       <c r="C51" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="E51" s="25" t="s">
+      <c r="E51" s="24" t="s">
         <v>65</v>
       </c>
       <c r="F51" s="1" t="s">
@@ -3341,34 +3479,34 @@
       </c>
     </row>
     <row r="54" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="33" t="s">
+      <c r="A54" s="32" t="s">
         <v>174</v>
       </c>
-      <c r="B54" s="22"/>
-      <c r="C54" s="23" t="s">
+      <c r="B54" s="21"/>
+      <c r="C54" s="22" t="s">
         <v>175</v>
       </c>
-      <c r="D54" s="23"/>
-      <c r="E54" s="22"/>
-      <c r="F54" s="22"/>
-      <c r="G54" s="22" t="s">
+      <c r="D54" s="22"/>
+      <c r="E54" s="21"/>
+      <c r="F54" s="21"/>
+      <c r="G54" s="21" t="s">
         <v>65</v>
       </c>
-      <c r="H54" s="23" t="s">
-        <v>15</v>
-      </c>
-      <c r="I54" s="23" t="str">
+      <c r="H54" s="22" t="s">
+        <v>15</v>
+      </c>
+      <c r="I54" s="22" t="str">
         <f aca="false">_xlfn.CONCAT(H54,"data_file")</f>
         <v>http://purl.org/ppeo/ppeo.owl#data_file</v>
       </c>
-      <c r="J54" s="22" t="str">
+      <c r="J54" s="21" t="str">
         <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G54)</f>
         <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#DataFile</v>
       </c>
-      <c r="K54" s="22"/>
+      <c r="K54" s="21"/>
     </row>
     <row r="55" s="13" customFormat="true" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="34"/>
+      <c r="A55" s="33"/>
       <c r="B55" s="14" t="s">
         <v>20</v>
       </c>
@@ -3397,7 +3535,7 @@
       </c>
     </row>
     <row r="56" s="13" customFormat="true" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="34"/>
+      <c r="A56" s="33"/>
       <c r="B56" s="14" t="s">
         <v>176</v>
       </c>
@@ -3426,7 +3564,7 @@
       </c>
     </row>
     <row r="57" s="13" customFormat="true" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="34"/>
+      <c r="A57" s="33"/>
       <c r="B57" s="14" t="s">
         <v>180</v>
       </c>
@@ -3455,7 +3593,7 @@
       </c>
     </row>
     <row r="58" s="13" customFormat="true" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="34"/>
+      <c r="A58" s="33"/>
       <c r="B58" s="14" t="s">
         <v>182</v>
       </c>
@@ -3484,7 +3622,7 @@
       </c>
     </row>
     <row r="59" s="13" customFormat="true" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="34"/>
+      <c r="A59" s="33"/>
       <c r="B59" s="14" t="s">
         <v>184</v>
       </c>
@@ -3513,14 +3651,14 @@
       </c>
     </row>
     <row r="60" s="13" customFormat="true" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="34"/>
+      <c r="A60" s="33"/>
       <c r="B60" s="14" t="s">
         <v>187</v>
       </c>
       <c r="C60" s="13" t="s">
         <v>188</v>
       </c>
-      <c r="E60" s="35" t="s">
+      <c r="E60" s="34" t="s">
         <v>189</v>
       </c>
       <c r="F60" s="13" t="s">
@@ -3542,7 +3680,7 @@
       </c>
     </row>
     <row r="61" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="26" t="s">
+      <c r="A61" s="25" t="s">
         <v>191</v>
       </c>
       <c r="B61" s="4"/>
@@ -3575,10 +3713,10 @@
       <c r="B62" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="C62" s="36" t="s">
+      <c r="C62" s="35" t="s">
         <v>141</v>
       </c>
-      <c r="D62" s="36"/>
+      <c r="D62" s="35"/>
       <c r="E62" s="1" t="s">
         <v>20</v>
       </c>
@@ -3605,8 +3743,8 @@
       <c r="B63" s="11" t="s">
         <v>195</v>
       </c>
-      <c r="C63" s="36"/>
-      <c r="D63" s="36"/>
+      <c r="C63" s="35"/>
+      <c r="D63" s="35"/>
       <c r="G63" s="13" t="s">
         <v>27</v>
       </c>
@@ -3627,8 +3765,8 @@
       <c r="B64" s="11" t="s">
         <v>196</v>
       </c>
-      <c r="C64" s="36"/>
-      <c r="D64" s="36"/>
+      <c r="C64" s="35"/>
+      <c r="D64" s="35"/>
       <c r="G64" s="13" t="s">
         <v>33</v>
       </c>
@@ -3649,11 +3787,11 @@
       <c r="B65" s="11" t="s">
         <v>197</v>
       </c>
-      <c r="C65" s="36" t="s">
+      <c r="C65" s="35" t="s">
         <v>198</v>
       </c>
-      <c r="D65" s="36"/>
-      <c r="G65" s="36" t="s">
+      <c r="D65" s="35"/>
+      <c r="G65" s="35" t="s">
         <v>199</v>
       </c>
       <c r="J65" s="1" t="str">
@@ -3666,8 +3804,8 @@
       <c r="B66" s="11" t="s">
         <v>200</v>
       </c>
-      <c r="C66" s="36"/>
-      <c r="D66" s="36"/>
+      <c r="C66" s="35"/>
+      <c r="D66" s="35"/>
       <c r="E66" s="1" t="s">
         <v>191</v>
       </c>
@@ -3691,8 +3829,8 @@
       <c r="B67" s="11" t="s">
         <v>202</v>
       </c>
-      <c r="C67" s="36"/>
-      <c r="D67" s="36"/>
+      <c r="C67" s="35"/>
+      <c r="D67" s="35"/>
       <c r="E67" s="1" t="s">
         <v>202</v>
       </c>
@@ -3716,17 +3854,17 @@
       <c r="B68" s="11" t="s">
         <v>205</v>
       </c>
-      <c r="C68" s="36" t="s">
+      <c r="C68" s="35" t="s">
         <v>206</v>
       </c>
-      <c r="D68" s="36"/>
+      <c r="D68" s="35"/>
       <c r="E68" s="1" t="s">
         <v>207</v>
       </c>
-      <c r="G68" s="36" t="s">
+      <c r="G68" s="35" t="s">
         <v>208</v>
       </c>
-      <c r="H68" s="36" t="s">
+      <c r="H68" s="35" t="s">
         <v>204</v>
       </c>
       <c r="I68" s="1" t="str">
@@ -3743,8 +3881,8 @@
       <c r="B69" s="11" t="s">
         <v>93</v>
       </c>
-      <c r="C69" s="36"/>
-      <c r="D69" s="36"/>
+      <c r="C69" s="35"/>
+      <c r="D69" s="35"/>
       <c r="E69" s="1" t="s">
         <v>93</v>
       </c>
@@ -3768,14 +3906,14 @@
       <c r="B70" s="11" t="s">
         <v>209</v>
       </c>
-      <c r="C70" s="36" t="s">
+      <c r="C70" s="35" t="s">
         <v>210</v>
       </c>
-      <c r="D70" s="36"/>
+      <c r="D70" s="35"/>
       <c r="E70" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="G70" s="36" t="s">
+      <c r="G70" s="35" t="s">
         <v>212</v>
       </c>
       <c r="I70" s="1" t="str">
@@ -3792,14 +3930,14 @@
       <c r="B71" s="11" t="s">
         <v>213</v>
       </c>
-      <c r="C71" s="36" t="s">
+      <c r="C71" s="35" t="s">
         <v>214</v>
       </c>
-      <c r="D71" s="36"/>
+      <c r="D71" s="35"/>
       <c r="E71" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="G71" s="36" t="s">
+      <c r="G71" s="35" t="s">
         <v>215</v>
       </c>
       <c r="I71" s="1" t="str">
@@ -3832,14 +3970,14 @@
       <c r="B73" s="11" t="s">
         <v>219</v>
       </c>
-      <c r="C73" s="36" t="s">
+      <c r="C73" s="35" t="s">
         <v>220</v>
       </c>
-      <c r="D73" s="36"/>
+      <c r="D73" s="35"/>
       <c r="E73" s="1" t="s">
         <v>221</v>
       </c>
-      <c r="G73" s="36"/>
+      <c r="G73" s="35"/>
       <c r="J73" s="1" t="str">
         <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G73)</f>
         <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#</v>
@@ -3946,34 +4084,34 @@
       </c>
     </row>
     <row r="84" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A84" s="33" t="s">
+      <c r="A84" s="32" t="s">
         <v>202</v>
       </c>
-      <c r="B84" s="22"/>
-      <c r="C84" s="23" t="s">
+      <c r="B84" s="21"/>
+      <c r="C84" s="22" t="s">
         <v>232</v>
       </c>
-      <c r="D84" s="23"/>
-      <c r="E84" s="22"/>
-      <c r="F84" s="22"/>
-      <c r="G84" s="22" t="s">
+      <c r="D84" s="22"/>
+      <c r="E84" s="21"/>
+      <c r="F84" s="21"/>
+      <c r="G84" s="21" t="s">
         <v>202</v>
       </c>
-      <c r="H84" s="23" t="s">
+      <c r="H84" s="22" t="s">
         <v>193</v>
       </c>
-      <c r="I84" s="23" t="str">
+      <c r="I84" s="22" t="str">
         <f aca="false">_xlfn.CONCAT(H84, G84)</f>
         <v>http://www.w3.org/ns/ssn/Platform</v>
       </c>
-      <c r="J84" s="22" t="str">
+      <c r="J84" s="21" t="str">
         <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G84)</f>
         <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#Platform</v>
       </c>
-      <c r="K84" s="22"/>
+      <c r="K84" s="21"/>
     </row>
     <row r="85" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A85" s="24"/>
+      <c r="A85" s="23"/>
       <c r="B85" s="11" t="s">
         <v>233</v>
       </c>
@@ -4002,7 +4140,7 @@
       </c>
     </row>
     <row r="86" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A86" s="24"/>
+      <c r="A86" s="23"/>
       <c r="B86" s="11" t="s">
         <v>234</v>
       </c>
@@ -4022,7 +4160,7 @@
       </c>
     </row>
     <row r="87" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A87" s="24"/>
+      <c r="A87" s="23"/>
       <c r="B87" s="11" t="s">
         <v>235</v>
       </c>
@@ -4042,7 +4180,7 @@
       </c>
     </row>
     <row r="88" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A88" s="24"/>
+      <c r="A88" s="23"/>
       <c r="B88" s="11" t="s">
         <v>236</v>
       </c>
@@ -4055,7 +4193,7 @@
       </c>
     </row>
     <row r="89" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A89" s="24"/>
+      <c r="A89" s="23"/>
       <c r="B89" s="11" t="s">
         <v>238</v>
       </c>
@@ -4068,7 +4206,7 @@
       </c>
     </row>
     <row r="90" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A90" s="24"/>
+      <c r="A90" s="23"/>
       <c r="B90" s="11" t="s">
         <v>240</v>
       </c>
@@ -4088,7 +4226,7 @@
       </c>
     </row>
     <row r="91" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A91" s="24"/>
+      <c r="A91" s="23"/>
       <c r="B91" s="11" t="s">
         <v>241</v>
       </c>
@@ -4101,7 +4239,7 @@
       </c>
     </row>
     <row r="92" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A92" s="26" t="s">
+      <c r="A92" s="25" t="s">
         <v>205</v>
       </c>
       <c r="B92" s="4"/>
@@ -4270,36 +4408,36 @@
       </c>
     </row>
     <row r="101" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A101" s="33" t="s">
+      <c r="A101" s="32" t="s">
         <v>248</v>
       </c>
-      <c r="B101" s="22"/>
-      <c r="C101" s="23" t="s">
+      <c r="B101" s="21"/>
+      <c r="C101" s="22" t="s">
         <v>250</v>
       </c>
-      <c r="D101" s="23"/>
-      <c r="E101" s="22"/>
-      <c r="F101" s="22"/>
-      <c r="G101" s="22" t="s">
+      <c r="D101" s="22"/>
+      <c r="E101" s="21"/>
+      <c r="F101" s="21"/>
+      <c r="G101" s="21" t="s">
         <v>251</v>
       </c>
-      <c r="H101" s="23" t="s">
+      <c r="H101" s="22" t="s">
         <v>204</v>
       </c>
-      <c r="I101" s="23" t="str">
+      <c r="I101" s="22" t="str">
         <f aca="false">_xlfn.CONCAT(H101, G101)</f>
         <v>http://www.w3.org/ns/sosa/Observation </v>
       </c>
-      <c r="J101" s="22" t="str">
+      <c r="J101" s="21" t="str">
         <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G101)</f>
         <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#Observation </v>
       </c>
-      <c r="K101" s="22" t="s">
+      <c r="K101" s="21" t="s">
         <v>194</v>
       </c>
     </row>
-    <row r="102" customFormat="false" ht="36.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A102" s="24"/>
+    <row r="102" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A102" s="23"/>
       <c r="B102" s="11" t="s">
         <v>20</v>
       </c>
@@ -4315,7 +4453,7 @@
       <c r="G102" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="H102" s="15" t="s">
+      <c r="H102" s="10" t="s">
         <v>15</v>
       </c>
       <c r="J102" s="1" t="str">
@@ -4323,15 +4461,15 @@
         <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#hasIdentifier</v>
       </c>
     </row>
-    <row r="103" customFormat="false" ht="36.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A103" s="24"/>
+    <row r="103" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A103" s="23"/>
       <c r="B103" s="11" t="s">
         <v>252</v>
       </c>
       <c r="G103" s="1" t="s">
         <v>253</v>
       </c>
-      <c r="H103" s="15" t="s">
+      <c r="H103" s="10" t="s">
         <v>15</v>
       </c>
       <c r="J103" s="1" t="str">
@@ -4340,7 +4478,7 @@
       </c>
     </row>
     <row r="104" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A104" s="24"/>
+      <c r="A104" s="23"/>
       <c r="B104" s="11" t="s">
         <v>254</v>
       </c>
@@ -4359,7 +4497,7 @@
       </c>
     </row>
     <row r="105" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A105" s="24"/>
+      <c r="A105" s="23"/>
       <c r="B105" s="11" t="s">
         <v>257</v>
       </c>
@@ -4375,7 +4513,7 @@
       </c>
     </row>
     <row r="106" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A106" s="24"/>
+      <c r="A106" s="23"/>
       <c r="B106" s="11" t="s">
         <v>259</v>
       </c>
@@ -4391,7 +4529,7 @@
       </c>
     </row>
     <row r="107" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A107" s="24"/>
+      <c r="A107" s="23"/>
       <c r="B107" s="11" t="s">
         <v>261</v>
       </c>
@@ -4407,7 +4545,7 @@
       </c>
     </row>
     <row r="108" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A108" s="26" t="s">
+      <c r="A108" s="25" t="s">
         <v>263</v>
       </c>
       <c r="B108" s="4"/>
@@ -4502,7 +4640,7 @@
       <c r="G111" s="1" t="s">
         <v>253</v>
       </c>
-      <c r="H111" s="15" t="s">
+      <c r="H111" s="10" t="s">
         <v>15</v>
       </c>
       <c r="I111" s="1" t="str">
@@ -4514,12 +4652,12 @@
         <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#partOf </v>
       </c>
     </row>
-    <row r="112" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="112" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="7"/>
       <c r="B112" s="11" t="s">
         <v>270</v>
       </c>
-      <c r="C112" s="15" t="s">
+      <c r="C112" s="10" t="s">
         <v>271</v>
       </c>
       <c r="G112" s="1" t="s">
@@ -4537,12 +4675,12 @@
         <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#hasDescription</v>
       </c>
     </row>
-    <row r="113" customFormat="false" ht="47.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="113" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="7"/>
       <c r="B113" s="11" t="s">
         <v>272</v>
       </c>
-      <c r="C113" s="15" t="s">
+      <c r="C113" s="10" t="s">
         <v>273</v>
       </c>
       <c r="G113" s="1" t="s">
@@ -4562,67 +4700,71 @@
     </row>
     <row r="114" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="7"/>
-      <c r="B114" s="27" t="s">
+      <c r="B114" s="26" t="s">
         <v>274</v>
       </c>
-      <c r="C114" s="28"/>
-      <c r="D114" s="28"/>
-      <c r="E114" s="28"/>
-      <c r="F114" s="28"/>
-      <c r="G114" s="28" t="s">
+      <c r="C114" s="27" t="s">
         <v>275</v>
       </c>
-      <c r="H114" s="28" t="s">
+      <c r="D114" s="27"/>
+      <c r="E114" s="27"/>
+      <c r="F114" s="27"/>
+      <c r="G114" s="27" t="s">
+        <v>276</v>
+      </c>
+      <c r="H114" s="27" t="s">
         <v>15</v>
       </c>
       <c r="I114" s="1" t="str">
         <f aca="false">_xlfn.CONCAT(H114,G114)</f>
         <v>http://purl.org/ppeo/ppeo.owl#hasSpatialDistribution</v>
       </c>
-      <c r="J114" s="28" t="str">
+      <c r="J114" s="27" t="str">
         <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G114)</f>
         <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#hasSpatialDistribution</v>
       </c>
-      <c r="K114" s="28"/>
+      <c r="K114" s="27"/>
       <c r="L114" s="1" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="7"/>
-      <c r="B115" s="27" t="s">
-        <v>277</v>
-      </c>
-      <c r="C115" s="28"/>
-      <c r="D115" s="28"/>
-      <c r="E115" s="28"/>
-      <c r="F115" s="28"/>
-      <c r="G115" s="28" t="s">
+      <c r="B115" s="26" t="s">
         <v>278</v>
       </c>
-      <c r="H115" s="28" t="s">
+      <c r="C115" s="27" t="s">
+        <v>279</v>
+      </c>
+      <c r="D115" s="27"/>
+      <c r="E115" s="27"/>
+      <c r="F115" s="27"/>
+      <c r="G115" s="27" t="s">
+        <v>280</v>
+      </c>
+      <c r="H115" s="27" t="s">
         <v>15</v>
       </c>
       <c r="I115" s="1" t="str">
         <f aca="false">_xlfn.CONCAT(H115,G115)</f>
         <v>http://purl.org/ppeo/ppeo.owl#hasSpatialDistributionType</v>
       </c>
-      <c r="J115" s="28" t="str">
+      <c r="J115" s="27" t="str">
         <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G115)</f>
         <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#hasSpatialDistributionType</v>
       </c>
-      <c r="K115" s="28"/>
+      <c r="K115" s="27"/>
     </row>
     <row r="116" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="7"/>
       <c r="B116" s="11" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="C116" s="1" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="D116" s="1" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="G116" s="1" t="s">
         <v>186</v>
@@ -4642,7 +4784,10 @@
     <row r="117" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="7"/>
       <c r="B117" s="11" t="s">
-        <v>282</v>
+        <v>284</v>
+      </c>
+      <c r="C117" s="1" t="s">
+        <v>285</v>
       </c>
       <c r="H117" s="10" t="s">
         <v>15</v>
@@ -4657,38 +4802,38 @@
       </c>
     </row>
     <row r="118" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A118" s="33" t="s">
-        <v>283</v>
-      </c>
-      <c r="B118" s="22"/>
-      <c r="C118" s="23" t="s">
-        <v>284</v>
-      </c>
-      <c r="D118" s="23"/>
-      <c r="E118" s="22"/>
-      <c r="F118" s="22"/>
-      <c r="G118" s="22" t="s">
-        <v>285</v>
-      </c>
-      <c r="H118" s="23" t="s">
-        <v>15</v>
-      </c>
-      <c r="I118" s="23" t="str">
+      <c r="A118" s="32" t="s">
+        <v>286</v>
+      </c>
+      <c r="B118" s="21"/>
+      <c r="C118" s="22" t="s">
+        <v>287</v>
+      </c>
+      <c r="D118" s="22"/>
+      <c r="E118" s="21"/>
+      <c r="F118" s="21"/>
+      <c r="G118" s="21" t="s">
+        <v>288</v>
+      </c>
+      <c r="H118" s="22" t="s">
+        <v>15</v>
+      </c>
+      <c r="I118" s="22" t="str">
         <f aca="false">_xlfn.CONCAT(H118,"observed_variable")</f>
         <v>http://purl.org/ppeo/ppeo.owl#observed_variable</v>
       </c>
-      <c r="J118" s="22" t="str">
+      <c r="J118" s="21" t="str">
         <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G118)</f>
         <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#ObservedVariable</v>
       </c>
-      <c r="K118" s="22" t="s">
-        <v>286</v>
+      <c r="K118" s="21" t="s">
+        <v>289</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A119" s="24"/>
+      <c r="A119" s="23"/>
       <c r="B119" s="11" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="C119" s="10" t="s">
         <v>141</v>
@@ -4704,10 +4849,16 @@
         <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#hasIdentifier</v>
       </c>
     </row>
-    <row r="120" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A120" s="24"/>
+    <row r="120" customFormat="false" ht="35.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A120" s="23"/>
       <c r="B120" s="11" t="s">
-        <v>288</v>
+        <v>291</v>
+      </c>
+      <c r="C120" s="1" t="s">
+        <v>292</v>
+      </c>
+      <c r="D120" s="10" t="s">
+        <v>293</v>
       </c>
       <c r="H120" s="10" t="s">
         <v>15</v>
@@ -4717,819 +4868,952 @@
         <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#</v>
       </c>
     </row>
-    <row r="121" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A121" s="24"/>
+    <row r="121" customFormat="false" ht="35.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A121" s="23"/>
       <c r="B121" s="11" t="s">
-        <v>289</v>
+        <v>294</v>
+      </c>
+      <c r="C121" s="1" t="s">
+        <v>295</v>
+      </c>
+      <c r="D121" s="10" t="s">
+        <v>296</v>
       </c>
       <c r="J121" s="1" t="str">
         <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G121)</f>
         <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#</v>
       </c>
     </row>
-    <row r="122" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A122" s="24"/>
+    <row r="122" customFormat="false" ht="35.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A122" s="23"/>
       <c r="B122" s="11" t="s">
-        <v>290</v>
+        <v>297</v>
+      </c>
+      <c r="C122" s="36" t="s">
+        <v>298</v>
+      </c>
+      <c r="D122" s="10" t="s">
+        <v>299</v>
       </c>
       <c r="J122" s="1" t="str">
         <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G122)</f>
         <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#</v>
       </c>
     </row>
-    <row r="123" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A123" s="24"/>
+    <row r="123" customFormat="false" ht="24.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A123" s="23"/>
       <c r="B123" s="11" t="s">
-        <v>291</v>
-      </c>
-    </row>
-    <row r="124" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A124" s="24"/>
+        <v>300</v>
+      </c>
+      <c r="C123" s="36" t="s">
+        <v>301</v>
+      </c>
+      <c r="D123" s="10" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="124" customFormat="false" ht="24.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A124" s="23"/>
       <c r="B124" s="11" t="s">
-        <v>292</v>
-      </c>
-    </row>
-    <row r="125" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A125" s="24"/>
-      <c r="B125" s="11"/>
-    </row>
-    <row r="126" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A126" s="24"/>
-      <c r="B126" s="11"/>
-      <c r="J126" s="1" t="str">
-        <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G126)</f>
+        <v>303</v>
+      </c>
+      <c r="C124" s="1" t="s">
+        <v>304</v>
+      </c>
+      <c r="D124" s="10" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="125" customFormat="false" ht="24.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A125" s="23"/>
+      <c r="B125" s="11" t="s">
+        <v>306</v>
+      </c>
+      <c r="C125" s="37" t="s">
+        <v>307</v>
+      </c>
+      <c r="D125" s="10" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="126" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A126" s="23"/>
+      <c r="B126" s="11" t="s">
+        <v>309</v>
+      </c>
+      <c r="D126" s="10" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="127" customFormat="false" ht="35.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A127" s="23"/>
+      <c r="B127" s="11" t="s">
+        <v>311</v>
+      </c>
+      <c r="C127" s="10" t="s">
+        <v>312</v>
+      </c>
+      <c r="D127" s="10" t="s">
+        <v>313</v>
+      </c>
+      <c r="J127" s="1" t="str">
+        <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G127)</f>
         <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#</v>
       </c>
     </row>
-    <row r="127" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A127" s="26" t="s">
-        <v>282</v>
-      </c>
-      <c r="B127" s="4"/>
-      <c r="C127" s="5" t="s">
-        <v>293</v>
-      </c>
-      <c r="D127" s="5"/>
-      <c r="E127" s="4"/>
-      <c r="F127" s="4"/>
-      <c r="G127" s="4" t="s">
-        <v>294</v>
-      </c>
-      <c r="H127" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="I127" s="5" t="str">
-        <f aca="false">_xlfn.CONCAT(H127,LOWER(G127))</f>
+    <row r="128" customFormat="false" ht="12.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A128" s="23"/>
+      <c r="B128" s="11" t="s">
+        <v>314</v>
+      </c>
+      <c r="C128" s="10" t="s">
+        <v>315</v>
+      </c>
+      <c r="D128" s="10" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="129" customFormat="false" ht="24.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A129" s="23"/>
+      <c r="B129" s="11" t="s">
+        <v>317</v>
+      </c>
+      <c r="C129" s="10" t="s">
+        <v>318</v>
+      </c>
+      <c r="D129" s="10" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="130" customFormat="false" ht="105.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A130" s="23"/>
+      <c r="B130" s="11" t="s">
+        <v>320</v>
+      </c>
+      <c r="C130" s="10" t="s">
+        <v>321</v>
+      </c>
+      <c r="D130" s="10" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="131" customFormat="false" ht="24.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A131" s="23"/>
+      <c r="B131" s="11" t="s">
+        <v>323</v>
+      </c>
+      <c r="C131" s="10" t="s">
+        <v>324</v>
+      </c>
+      <c r="D131" s="10" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="132" customFormat="false" ht="12.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A132" s="23"/>
+      <c r="B132" s="11" t="s">
+        <v>326</v>
+      </c>
+      <c r="C132" s="10" t="s">
+        <v>327</v>
+      </c>
+      <c r="D132" s="10" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="133" customFormat="false" ht="24.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A133" s="23"/>
+      <c r="B133" s="11" t="s">
+        <v>329</v>
+      </c>
+      <c r="C133" s="10" t="s">
+        <v>330</v>
+      </c>
+      <c r="D133" s="10" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="134" customFormat="false" ht="24.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A134" s="23"/>
+      <c r="B134" s="11" t="s">
+        <v>332</v>
+      </c>
+      <c r="C134" s="10" t="s">
+        <v>333</v>
+      </c>
+      <c r="D134" s="10" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="135" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A135" s="25" t="s">
+        <v>284</v>
+      </c>
+      <c r="B135" s="4"/>
+      <c r="C135" s="5" t="s">
+        <v>335</v>
+      </c>
+      <c r="D135" s="5"/>
+      <c r="E135" s="4"/>
+      <c r="F135" s="4"/>
+      <c r="G135" s="4" t="s">
+        <v>336</v>
+      </c>
+      <c r="H135" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="I135" s="5" t="str">
+        <f aca="false">_xlfn.CONCAT(H135,LOWER(G135))</f>
         <v>http://purl.org/ppeo/ppeo.owl#factor</v>
       </c>
-      <c r="J127" s="4" t="str">
-        <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G127)</f>
+      <c r="J135" s="4" t="str">
+        <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G135)</f>
         <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#Factor</v>
       </c>
-      <c r="K127" s="4"/>
-    </row>
-    <row r="128" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A128" s="7"/>
-      <c r="B128" s="11" t="s">
+      <c r="K135" s="4"/>
+    </row>
+    <row r="136" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A136" s="7"/>
+      <c r="B136" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="C128" s="10" t="s">
+      <c r="C136" s="10" t="s">
         <v>141</v>
       </c>
-      <c r="G128" s="1" t="s">
+      <c r="G136" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="H128" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="J128" s="1" t="str">
-        <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G128)</f>
+      <c r="H136" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="J136" s="1" t="str">
+        <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G136)</f>
         <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#hasIdentifier</v>
       </c>
     </row>
-    <row r="129" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A129" s="7"/>
-      <c r="B129" s="11" t="s">
+    <row r="137" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A137" s="7"/>
+      <c r="B137" s="11" t="s">
         <v>252</v>
       </c>
-      <c r="G129" s="1" t="s">
+      <c r="G137" s="1" t="s">
         <v>253</v>
       </c>
-      <c r="J129" s="1" t="str">
-        <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G129)</f>
-        <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#partOf </v>
-      </c>
-    </row>
-    <row r="130" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A130" s="7"/>
-      <c r="B130" s="11" t="s">
-        <v>295</v>
-      </c>
-      <c r="J130" s="1" t="str">
-        <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G130)</f>
-        <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#</v>
-      </c>
-    </row>
-    <row r="131" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A131" s="7"/>
-      <c r="B131" s="11" t="s">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="132" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A132" s="7"/>
-      <c r="B132" s="11" t="s">
-        <v>297</v>
-      </c>
-    </row>
-    <row r="133" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A133" s="7"/>
-      <c r="B133" s="11" t="s">
-        <v>298</v>
-      </c>
-      <c r="C133" s="1" t="s">
-        <v>299</v>
-      </c>
-    </row>
-    <row r="134" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A134" s="33" t="s">
-        <v>300</v>
-      </c>
-      <c r="B134" s="22"/>
-      <c r="C134" s="23" t="s">
-        <v>301</v>
-      </c>
-      <c r="D134" s="23"/>
-      <c r="E134" s="22"/>
-      <c r="F134" s="22"/>
-      <c r="G134" s="22" t="s">
-        <v>300</v>
-      </c>
-      <c r="H134" s="23" t="s">
-        <v>15</v>
-      </c>
-      <c r="I134" s="23"/>
-      <c r="J134" s="22" t="str">
-        <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G134)</f>
-        <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#Sample</v>
-      </c>
-      <c r="K134" s="22"/>
-    </row>
-    <row r="135" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A135" s="24"/>
-      <c r="B135" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="C135" s="10" t="s">
-        <v>141</v>
-      </c>
-      <c r="G135" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="H135" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="J135" s="1" t="str">
-        <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G135)</f>
-        <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#hasIdentifier</v>
-      </c>
-    </row>
-    <row r="136" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A136" s="24"/>
-      <c r="B136" s="11"/>
-      <c r="C136" s="10"/>
-    </row>
-    <row r="137" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A137" s="24"/>
-      <c r="B137" s="11"/>
       <c r="J137" s="1" t="str">
         <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G137)</f>
+        <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#partOf </v>
+      </c>
+    </row>
+    <row r="138" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A138" s="7"/>
+      <c r="B138" s="11" t="s">
+        <v>337</v>
+      </c>
+      <c r="J138" s="1" t="str">
+        <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G138)</f>
         <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#</v>
       </c>
     </row>
-    <row r="138" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A138" s="26" t="s">
-        <v>302</v>
-      </c>
-      <c r="B138" s="4"/>
-      <c r="C138" s="5" t="s">
-        <v>303</v>
-      </c>
-      <c r="D138" s="5"/>
-      <c r="E138" s="4"/>
-      <c r="F138" s="4"/>
-      <c r="G138" s="4" t="s">
-        <v>304</v>
-      </c>
-      <c r="H138" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="I138" s="5"/>
-      <c r="J138" s="4" t="str">
-        <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G138)</f>
-        <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#BiologicalMaterial</v>
-      </c>
-      <c r="K138" s="4"/>
-    </row>
-    <row r="139" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="139" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A139" s="7"/>
       <c r="B139" s="11" t="s">
-        <v>305</v>
-      </c>
-      <c r="C139" s="10" t="s">
-        <v>306</v>
-      </c>
-      <c r="G139" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="H139" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="J139" s="1" t="str">
-        <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G139)</f>
-        <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#hasIdentifier</v>
-      </c>
-    </row>
-    <row r="140" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="140" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A140" s="7"/>
       <c r="B140" s="11" t="s">
-        <v>307</v>
-      </c>
-      <c r="C140" s="1" t="s">
-        <v>308</v>
-      </c>
-      <c r="J140" s="1" t="str">
-        <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G140)</f>
-        <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#</v>
+        <v>339</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A141" s="7"/>
       <c r="B141" s="11" t="s">
-        <v>309</v>
+        <v>340</v>
       </c>
       <c r="C141" s="1" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="142" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A142" s="7"/>
-      <c r="B142" s="11" t="s">
-        <v>311</v>
-      </c>
-    </row>
-    <row r="143" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A143" s="7"/>
+        <v>341</v>
+      </c>
+    </row>
+    <row r="142" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A142" s="32" t="s">
+        <v>342</v>
+      </c>
+      <c r="B142" s="21"/>
+      <c r="C142" s="22" t="s">
+        <v>343</v>
+      </c>
+      <c r="D142" s="22"/>
+      <c r="E142" s="21"/>
+      <c r="F142" s="21"/>
+      <c r="G142" s="21" t="s">
+        <v>342</v>
+      </c>
+      <c r="H142" s="22" t="s">
+        <v>15</v>
+      </c>
+      <c r="I142" s="22"/>
+      <c r="J142" s="21" t="str">
+        <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G142)</f>
+        <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#Sample</v>
+      </c>
+      <c r="K142" s="21"/>
+    </row>
+    <row r="143" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A143" s="23"/>
       <c r="B143" s="11" t="s">
-        <v>312</v>
+        <v>20</v>
+      </c>
+      <c r="C143" s="10" t="s">
+        <v>141</v>
+      </c>
+      <c r="G143" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H143" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="J143" s="1" t="str">
+        <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G143)</f>
+        <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#hasIdentifier</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A144" s="7"/>
-      <c r="B144" s="11" t="s">
-        <v>313</v>
-      </c>
-    </row>
-    <row r="145" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A145" s="7"/>
+      <c r="A144" s="23"/>
+      <c r="B144" s="11"/>
+      <c r="C144" s="10"/>
+    </row>
+    <row r="145" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A145" s="23"/>
       <c r="B145" s="11"/>
-    </row>
-    <row r="146" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A146" s="7"/>
-      <c r="B146" s="11"/>
-    </row>
-    <row r="147" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="J145" s="1" t="str">
+        <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G145)</f>
+        <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#</v>
+      </c>
+    </row>
+    <row r="146" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A146" s="25" t="s">
+        <v>344</v>
+      </c>
+      <c r="B146" s="4"/>
+      <c r="C146" s="5" t="s">
+        <v>345</v>
+      </c>
+      <c r="D146" s="5"/>
+      <c r="E146" s="4"/>
+      <c r="F146" s="4"/>
+      <c r="G146" s="4" t="s">
+        <v>346</v>
+      </c>
+      <c r="H146" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="I146" s="5"/>
+      <c r="J146" s="4" t="str">
+        <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G146)</f>
+        <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#BiologicalMaterial</v>
+      </c>
+      <c r="K146" s="4"/>
+    </row>
+    <row r="147" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A147" s="7"/>
-      <c r="B147" s="11"/>
-    </row>
-    <row r="148" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B147" s="11" t="s">
+        <v>347</v>
+      </c>
+      <c r="C147" s="10" t="s">
+        <v>348</v>
+      </c>
+      <c r="G147" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H147" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="J147" s="1" t="str">
+        <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G147)</f>
+        <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#hasIdentifier</v>
+      </c>
+    </row>
+    <row r="148" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A148" s="7"/>
-      <c r="B148" s="11"/>
-    </row>
-    <row r="149" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B148" s="11" t="s">
+        <v>349</v>
+      </c>
+      <c r="C148" s="1" t="s">
+        <v>350</v>
+      </c>
+      <c r="J148" s="1" t="str">
+        <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G148)</f>
+        <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#</v>
+      </c>
+    </row>
+    <row r="149" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A149" s="7"/>
-      <c r="B149" s="11"/>
+      <c r="B149" s="11" t="s">
+        <v>351</v>
+      </c>
+      <c r="C149" s="1" t="s">
+        <v>352</v>
+      </c>
     </row>
     <row r="150" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A150" s="7"/>
-      <c r="B150" s="11"/>
+      <c r="B150" s="11" t="s">
+        <v>353</v>
+      </c>
     </row>
     <row r="151" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A151" s="7"/>
-      <c r="B151" s="11"/>
+      <c r="B151" s="11" t="s">
+        <v>354</v>
+      </c>
     </row>
     <row r="152" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A152" s="7"/>
-      <c r="B152" s="11"/>
-    </row>
-    <row r="153" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A153" s="33" t="s">
-        <v>314</v>
-      </c>
-      <c r="B153" s="22"/>
-      <c r="C153" s="23" t="s">
-        <v>315</v>
-      </c>
-      <c r="D153" s="23"/>
-      <c r="E153" s="22"/>
-      <c r="F153" s="22"/>
-      <c r="G153" s="22" t="s">
-        <v>314</v>
-      </c>
-      <c r="H153" s="23" t="s">
-        <v>15</v>
-      </c>
-      <c r="I153" s="23"/>
-      <c r="J153" s="22" t="str">
-        <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G153)</f>
+      <c r="B152" s="11" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="153" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A153" s="7"/>
+      <c r="B153" s="11"/>
+    </row>
+    <row r="154" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A154" s="7"/>
+      <c r="B154" s="11"/>
+    </row>
+    <row r="155" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A155" s="7"/>
+      <c r="B155" s="11"/>
+    </row>
+    <row r="156" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A156" s="7"/>
+      <c r="B156" s="11"/>
+    </row>
+    <row r="157" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A157" s="7"/>
+      <c r="B157" s="11"/>
+    </row>
+    <row r="158" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A158" s="7"/>
+      <c r="B158" s="11"/>
+    </row>
+    <row r="159" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A159" s="7"/>
+      <c r="B159" s="11"/>
+    </row>
+    <row r="160" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A160" s="7"/>
+      <c r="B160" s="11"/>
+    </row>
+    <row r="161" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A161" s="32" t="s">
+        <v>356</v>
+      </c>
+      <c r="B161" s="21"/>
+      <c r="C161" s="22" t="s">
+        <v>357</v>
+      </c>
+      <c r="D161" s="22"/>
+      <c r="E161" s="21"/>
+      <c r="F161" s="21"/>
+      <c r="G161" s="21" t="s">
+        <v>356</v>
+      </c>
+      <c r="H161" s="22" t="s">
+        <v>15</v>
+      </c>
+      <c r="I161" s="22"/>
+      <c r="J161" s="21" t="str">
+        <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G161)</f>
         <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#Event</v>
       </c>
-      <c r="K153" s="22"/>
-    </row>
-    <row r="154" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A154" s="24"/>
-      <c r="B154" s="11" t="s">
+      <c r="K161" s="21"/>
+    </row>
+    <row r="162" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A162" s="23"/>
+      <c r="B162" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="C154" s="10" t="s">
+      <c r="C162" s="10" t="s">
         <v>141</v>
       </c>
-      <c r="G154" s="1" t="s">
+      <c r="G162" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="H154" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="J154" s="1" t="str">
-        <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G154)</f>
+      <c r="H162" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="J162" s="1" t="str">
+        <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G162)</f>
         <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#hasIdentifier</v>
       </c>
     </row>
-    <row r="155" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A155" s="24"/>
-      <c r="B155" s="11"/>
-      <c r="J155" s="1" t="str">
-        <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G155)</f>
+    <row r="163" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A163" s="23"/>
+      <c r="B163" s="11"/>
+      <c r="J163" s="1" t="str">
+        <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G163)</f>
         <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#</v>
       </c>
     </row>
-    <row r="156" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A156" s="24"/>
-      <c r="B156" s="11"/>
-      <c r="J156" s="1" t="str">
-        <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G156)</f>
+    <row r="164" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A164" s="23"/>
+      <c r="B164" s="11"/>
+      <c r="J164" s="1" t="str">
+        <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G164)</f>
         <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#</v>
       </c>
     </row>
-    <row r="157" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A157" s="24"/>
-      <c r="B157" s="11"/>
-      <c r="J157" s="1" t="str">
-        <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G157)</f>
-        <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#</v>
-      </c>
-    </row>
-    <row r="158" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A158" s="26" t="s">
-        <v>316</v>
-      </c>
-      <c r="B158" s="4"/>
-      <c r="C158" s="5" t="s">
-        <v>317</v>
-      </c>
-      <c r="D158" s="5"/>
-      <c r="E158" s="4"/>
-      <c r="F158" s="4"/>
-      <c r="G158" s="4"/>
-      <c r="H158" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="I158" s="5"/>
-      <c r="J158" s="4" t="str">
-        <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G158)</f>
-        <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#</v>
-      </c>
-      <c r="K158" s="4"/>
-    </row>
-    <row r="159" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A159" s="7"/>
-      <c r="B159" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="C159" s="10" t="s">
-        <v>141</v>
-      </c>
-      <c r="G159" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="H159" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="J159" s="1" t="str">
-        <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G159)</f>
-        <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#hasIdentifier</v>
-      </c>
-    </row>
-    <row r="160" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A160" s="7"/>
-      <c r="B160" s="11" t="s">
-        <v>68</v>
-      </c>
-      <c r="C160" s="10" t="s">
-        <v>318</v>
-      </c>
-      <c r="E160" s="1" t="s">
-        <v>319</v>
-      </c>
-      <c r="G160" s="1" t="s">
-        <v>190</v>
-      </c>
-      <c r="H160" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="K160" s="1" t="s">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="161" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A161" s="7"/>
-      <c r="B161" s="11" t="s">
-        <v>321</v>
-      </c>
-      <c r="C161" s="1" t="s">
-        <v>322</v>
-      </c>
-      <c r="E161" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="G161" s="1" t="s">
-        <v>323</v>
-      </c>
-      <c r="H161" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="J161" s="1" t="str">
-        <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G161)</f>
-        <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#hasEnvironmentParameter</v>
-      </c>
-    </row>
-    <row r="162" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A162" s="7"/>
-      <c r="B162" s="11" t="s">
-        <v>324</v>
-      </c>
-      <c r="C162" s="1" t="s">
-        <v>325</v>
-      </c>
-      <c r="E162" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="G162" s="1" t="s">
-        <v>326</v>
-      </c>
-      <c r="H162" s="10" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="163" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A163" s="7"/>
-      <c r="B163" s="11" t="s">
-        <v>298</v>
-      </c>
-      <c r="C163" s="1" t="s">
-        <v>299</v>
-      </c>
-      <c r="E163" s="1" t="s">
-        <v>174</v>
-      </c>
-      <c r="F163" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="G163" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="H163" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="164" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A164" s="33" t="s">
-        <v>327</v>
-      </c>
-      <c r="B164" s="22"/>
-      <c r="C164" s="23" t="s">
-        <v>328</v>
-      </c>
-      <c r="D164" s="23"/>
-      <c r="E164" s="22"/>
-      <c r="F164" s="22" t="s">
-        <v>70</v>
-      </c>
-      <c r="G164" s="22" t="s">
-        <v>327</v>
-      </c>
-      <c r="H164" s="23" t="s">
-        <v>15</v>
-      </c>
-      <c r="I164" s="23"/>
-      <c r="J164" s="22" t="str">
-        <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G164)</f>
-        <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#Person</v>
-      </c>
-      <c r="K164" s="22"/>
-    </row>
-    <row r="165" s="31" customFormat="true" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A165" s="24"/>
-      <c r="B165" s="11" t="s">
-        <v>329</v>
-      </c>
-      <c r="C165" s="1" t="s">
-        <v>141</v>
-      </c>
-      <c r="E165" s="31" t="s">
-        <v>20</v>
-      </c>
-      <c r="F165" s="31" t="s">
-        <v>14</v>
-      </c>
-      <c r="G165" s="31" t="s">
-        <v>21</v>
-      </c>
-      <c r="H165" s="37" t="s">
-        <v>15</v>
-      </c>
+    <row r="165" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A165" s="23"/>
+      <c r="B165" s="11"/>
       <c r="J165" s="1" t="str">
         <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G165)</f>
-        <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#hasIdentifier</v>
-      </c>
-    </row>
-    <row r="166" s="31" customFormat="true" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A166" s="24"/>
-      <c r="B166" s="11" t="s">
-        <v>330</v>
-      </c>
-      <c r="C166" s="1" t="s">
-        <v>331</v>
-      </c>
-      <c r="E166" s="31" t="s">
-        <v>26</v>
-      </c>
-      <c r="F166" s="31" t="s">
-        <v>14</v>
-      </c>
-      <c r="G166" s="31" t="s">
-        <v>27</v>
-      </c>
-      <c r="H166" s="37" t="s">
-        <v>15</v>
-      </c>
-      <c r="J166" s="1" t="str">
+        <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#</v>
+      </c>
+    </row>
+    <row r="166" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A166" s="25" t="s">
+        <v>358</v>
+      </c>
+      <c r="B166" s="4"/>
+      <c r="C166" s="5" t="s">
+        <v>359</v>
+      </c>
+      <c r="D166" s="5"/>
+      <c r="E166" s="4"/>
+      <c r="F166" s="4"/>
+      <c r="G166" s="4"/>
+      <c r="H166" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="I166" s="5"/>
+      <c r="J166" s="4" t="str">
         <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G166)</f>
-        <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#hasName</v>
-      </c>
-    </row>
-    <row r="167" s="31" customFormat="true" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A167" s="24"/>
+        <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#</v>
+      </c>
+      <c r="K166" s="4"/>
+    </row>
+    <row r="167" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A167" s="7"/>
       <c r="B167" s="11" t="s">
-        <v>332</v>
-      </c>
-      <c r="C167" s="1" t="s">
-        <v>333</v>
-      </c>
-      <c r="E167" s="31" t="s">
         <v>20</v>
       </c>
-      <c r="F167" s="31" t="s">
-        <v>66</v>
-      </c>
-      <c r="G167" s="31" t="s">
-        <v>334</v>
-      </c>
-      <c r="H167" s="37" t="s">
+      <c r="C167" s="10" t="s">
+        <v>141</v>
+      </c>
+      <c r="G167" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H167" s="10" t="s">
         <v>15</v>
       </c>
       <c r="J167" s="1" t="str">
         <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G167)</f>
-        <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#hasORCID</v>
-      </c>
-    </row>
-    <row r="168" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A168" s="24"/>
+        <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#hasIdentifier</v>
+      </c>
+    </row>
+    <row r="168" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A168" s="7"/>
       <c r="B168" s="11" t="s">
-        <v>335</v>
-      </c>
-      <c r="C168" s="1" t="s">
-        <v>336</v>
-      </c>
-      <c r="D168" s="31"/>
+        <v>68</v>
+      </c>
+      <c r="C168" s="10" t="s">
+        <v>360</v>
+      </c>
       <c r="E168" s="1" t="s">
+        <v>361</v>
+      </c>
+      <c r="G168" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="H168" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="K168" s="1" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="169" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A169" s="7"/>
+      <c r="B169" s="11" t="s">
+        <v>363</v>
+      </c>
+      <c r="C169" s="1" t="s">
+        <v>364</v>
+      </c>
+      <c r="E169" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="F168" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="G168" s="1" t="s">
-        <v>337</v>
-      </c>
-      <c r="H168" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="J168" s="1" t="str">
-        <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G168)</f>
-        <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#hasEmailContact</v>
-      </c>
-    </row>
-    <row r="169" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A169" s="24"/>
-      <c r="B169" s="11" t="s">
-        <v>338</v>
-      </c>
-      <c r="C169" s="1" t="s">
-        <v>339</v>
-      </c>
-      <c r="E169" s="25" t="s">
-        <v>338</v>
-      </c>
-      <c r="F169" s="1" t="s">
-        <v>66</v>
-      </c>
       <c r="G169" s="1" t="s">
-        <v>340</v>
+        <v>365</v>
       </c>
       <c r="H169" s="10" t="s">
         <v>15</v>
       </c>
       <c r="J169" s="1" t="str">
         <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G169)</f>
-        <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#hasRole</v>
-      </c>
-    </row>
-    <row r="170" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A170" s="24"/>
+        <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#hasEnvironmentParameter</v>
+      </c>
+    </row>
+    <row r="170" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A170" s="7"/>
       <c r="B170" s="11" t="s">
+        <v>366</v>
+      </c>
+      <c r="C170" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="E170" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="G170" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="H170" s="10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="171" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A171" s="7"/>
+      <c r="B171" s="11" t="s">
+        <v>340</v>
+      </c>
+      <c r="C171" s="1" t="s">
         <v>341</v>
       </c>
-      <c r="C170" s="1" t="s">
-        <v>342</v>
-      </c>
-      <c r="E170" s="25" t="s">
-        <v>91</v>
-      </c>
-      <c r="F170" s="1" t="s">
+      <c r="E171" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="F171" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="G171" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="H171" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="172" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A172" s="32" t="s">
+        <v>369</v>
+      </c>
+      <c r="B172" s="21"/>
+      <c r="C172" s="22" t="s">
+        <v>370</v>
+      </c>
+      <c r="D172" s="22"/>
+      <c r="E172" s="21"/>
+      <c r="F172" s="21" t="s">
         <v>70</v>
       </c>
-      <c r="G170" s="1" t="s">
-        <v>343</v>
-      </c>
-      <c r="H170" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="J170" s="1" t="str">
-        <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G170)</f>
-        <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#hasAffiliation</v>
-      </c>
-    </row>
-    <row r="171" customFormat="false" ht="147" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A171" s="38" t="s">
-        <v>344</v>
-      </c>
-      <c r="B171" s="39"/>
-      <c r="C171" s="40" t="s">
-        <v>345</v>
-      </c>
-      <c r="D171" s="40"/>
-      <c r="E171" s="39"/>
-      <c r="F171" s="39"/>
-      <c r="G171" s="39"/>
-      <c r="H171" s="40"/>
-      <c r="I171" s="40"/>
-      <c r="J171" s="39" t="str">
-        <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G171)</f>
-        <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#</v>
-      </c>
-      <c r="K171" s="39" t="s">
-        <v>346</v>
-      </c>
-    </row>
-    <row r="172" s="13" customFormat="true" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A172" s="41"/>
-      <c r="B172" s="14" t="s">
+      <c r="G172" s="21" t="s">
+        <v>369</v>
+      </c>
+      <c r="H172" s="22" t="s">
+        <v>15</v>
+      </c>
+      <c r="I172" s="22"/>
+      <c r="J172" s="21" t="str">
+        <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G172)</f>
+        <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#Person</v>
+      </c>
+      <c r="K172" s="21"/>
+    </row>
+    <row r="173" s="30" customFormat="true" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A173" s="23"/>
+      <c r="B173" s="11" t="s">
+        <v>371</v>
+      </c>
+      <c r="C173" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="E173" s="30" t="s">
         <v>20</v>
       </c>
-      <c r="C172" s="13" t="s">
-        <v>141</v>
-      </c>
-      <c r="J172" s="1" t="str">
-        <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G172)</f>
-        <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#</v>
-      </c>
-    </row>
-    <row r="173" s="13" customFormat="true" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A173" s="41"/>
-      <c r="B173" s="14" t="s">
-        <v>347</v>
+      <c r="F173" s="30" t="s">
+        <v>14</v>
+      </c>
+      <c r="G173" s="30" t="s">
+        <v>21</v>
+      </c>
+      <c r="H173" s="38" t="s">
+        <v>15</v>
       </c>
       <c r="J173" s="1" t="str">
         <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G173)</f>
-        <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#</v>
-      </c>
-    </row>
-    <row r="174" s="13" customFormat="true" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A174" s="41"/>
-      <c r="B174" s="14" t="s">
-        <v>348</v>
+        <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#hasIdentifier</v>
+      </c>
+    </row>
+    <row r="174" s="30" customFormat="true" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A174" s="23"/>
+      <c r="B174" s="11" t="s">
+        <v>372</v>
+      </c>
+      <c r="C174" s="1" t="s">
+        <v>373</v>
+      </c>
+      <c r="E174" s="30" t="s">
+        <v>26</v>
+      </c>
+      <c r="F174" s="30" t="s">
+        <v>14</v>
+      </c>
+      <c r="G174" s="30" t="s">
+        <v>27</v>
+      </c>
+      <c r="H174" s="38" t="s">
+        <v>15</v>
       </c>
       <c r="J174" s="1" t="str">
         <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G174)</f>
-        <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#</v>
-      </c>
-    </row>
-    <row r="175" s="13" customFormat="true" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A175" s="41"/>
-      <c r="B175" s="14" t="s">
-        <v>209</v>
+        <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#hasName</v>
+      </c>
+    </row>
+    <row r="175" s="30" customFormat="true" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A175" s="23"/>
+      <c r="B175" s="11" t="s">
+        <v>374</v>
+      </c>
+      <c r="C175" s="1" t="s">
+        <v>375</v>
+      </c>
+      <c r="E175" s="30" t="s">
+        <v>20</v>
+      </c>
+      <c r="F175" s="30" t="s">
+        <v>66</v>
+      </c>
+      <c r="G175" s="30" t="s">
+        <v>376</v>
+      </c>
+      <c r="H175" s="38" t="s">
+        <v>15</v>
       </c>
       <c r="J175" s="1" t="str">
         <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G175)</f>
-        <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#</v>
-      </c>
-    </row>
-    <row r="176" s="13" customFormat="true" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A176" s="41"/>
-      <c r="B176" s="14" t="s">
-        <v>213</v>
+        <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#hasORCID</v>
+      </c>
+    </row>
+    <row r="176" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A176" s="23"/>
+      <c r="B176" s="11" t="s">
+        <v>377</v>
+      </c>
+      <c r="C176" s="1" t="s">
+        <v>378</v>
+      </c>
+      <c r="D176" s="30"/>
+      <c r="E176" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="F176" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="G176" s="1" t="s">
+        <v>379</v>
+      </c>
+      <c r="H176" s="10" t="s">
+        <v>15</v>
       </c>
       <c r="J176" s="1" t="str">
         <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G176)</f>
-        <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#</v>
-      </c>
-    </row>
-    <row r="177" s="13" customFormat="true" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A177" s="41"/>
-      <c r="B177" s="14" t="s">
-        <v>349</v>
+        <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#hasEmailContact</v>
+      </c>
+    </row>
+    <row r="177" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A177" s="23"/>
+      <c r="B177" s="11" t="s">
+        <v>380</v>
+      </c>
+      <c r="C177" s="1" t="s">
+        <v>381</v>
+      </c>
+      <c r="E177" s="24" t="s">
+        <v>380</v>
+      </c>
+      <c r="F177" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="G177" s="1" t="s">
+        <v>382</v>
+      </c>
+      <c r="H177" s="10" t="s">
+        <v>15</v>
       </c>
       <c r="J177" s="1" t="str">
         <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G177)</f>
-        <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#</v>
-      </c>
-    </row>
-    <row r="178" s="13" customFormat="true" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A178" s="41"/>
-      <c r="B178" s="14" t="s">
-        <v>350</v>
-      </c>
-      <c r="E178" s="13" t="s">
-        <v>351</v>
+        <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#hasRole</v>
+      </c>
+    </row>
+    <row r="178" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A178" s="23"/>
+      <c r="B178" s="11" t="s">
+        <v>383</v>
+      </c>
+      <c r="C178" s="1" t="s">
+        <v>384</v>
+      </c>
+      <c r="E178" s="24" t="s">
+        <v>91</v>
+      </c>
+      <c r="F178" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="G178" s="1" t="s">
+        <v>385</v>
+      </c>
+      <c r="H178" s="10" t="s">
+        <v>15</v>
       </c>
       <c r="J178" s="1" t="str">
         <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G178)</f>
-        <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#</v>
-      </c>
-    </row>
-    <row r="179" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A179" s="38" t="s">
-        <v>352</v>
-      </c>
-      <c r="B179" s="39"/>
-      <c r="C179" s="40" t="s">
-        <v>353</v>
-      </c>
-      <c r="D179" s="40"/>
-      <c r="E179" s="39"/>
-      <c r="F179" s="39"/>
-      <c r="G179" s="39"/>
-      <c r="H179" s="40"/>
-      <c r="I179" s="40"/>
-      <c r="J179" s="39" t="str">
+        <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#hasAffiliation</v>
+      </c>
+    </row>
+    <row r="179" customFormat="false" ht="147" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A179" s="39" t="s">
+        <v>386</v>
+      </c>
+      <c r="B179" s="40"/>
+      <c r="C179" s="41" t="s">
+        <v>387</v>
+      </c>
+      <c r="D179" s="41"/>
+      <c r="E179" s="40"/>
+      <c r="F179" s="40"/>
+      <c r="G179" s="40"/>
+      <c r="H179" s="41"/>
+      <c r="I179" s="41"/>
+      <c r="J179" s="40" t="str">
         <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G179)</f>
         <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#</v>
       </c>
-      <c r="K179" s="39" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="180" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A180" s="41"/>
-      <c r="B180" s="11" t="s">
+      <c r="K179" s="40" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="180" s="13" customFormat="true" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A180" s="42"/>
+      <c r="B180" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="C180" s="10" t="s">
+      <c r="C180" s="13" t="s">
         <v>141</v>
-      </c>
-      <c r="G180" s="1" t="s">
-        <v>21</v>
       </c>
       <c r="J180" s="1" t="str">
         <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G180)</f>
-        <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#hasIdentifier</v>
-      </c>
-    </row>
-    <row r="181" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A181" s="41"/>
-      <c r="B181" s="11"/>
+        <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#</v>
+      </c>
+    </row>
+    <row r="181" s="13" customFormat="true" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A181" s="42"/>
+      <c r="B181" s="14" t="s">
+        <v>389</v>
+      </c>
       <c r="J181" s="1" t="str">
         <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G181)</f>
+        <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#</v>
+      </c>
+    </row>
+    <row r="182" s="13" customFormat="true" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A182" s="42"/>
+      <c r="B182" s="14" t="s">
+        <v>390</v>
+      </c>
+      <c r="J182" s="1" t="str">
+        <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G182)</f>
+        <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#</v>
+      </c>
+    </row>
+    <row r="183" s="13" customFormat="true" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A183" s="42"/>
+      <c r="B183" s="14" t="s">
+        <v>209</v>
+      </c>
+      <c r="J183" s="1" t="str">
+        <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G183)</f>
+        <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#</v>
+      </c>
+    </row>
+    <row r="184" s="13" customFormat="true" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A184" s="42"/>
+      <c r="B184" s="14" t="s">
+        <v>213</v>
+      </c>
+      <c r="J184" s="1" t="str">
+        <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G184)</f>
+        <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#</v>
+      </c>
+    </row>
+    <row r="185" s="13" customFormat="true" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A185" s="42"/>
+      <c r="B185" s="14" t="s">
+        <v>391</v>
+      </c>
+      <c r="J185" s="1" t="str">
+        <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G185)</f>
+        <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#</v>
+      </c>
+    </row>
+    <row r="186" s="13" customFormat="true" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A186" s="42"/>
+      <c r="B186" s="14" t="s">
+        <v>392</v>
+      </c>
+      <c r="E186" s="13" t="s">
+        <v>393</v>
+      </c>
+      <c r="J186" s="1" t="str">
+        <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G186)</f>
+        <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#</v>
+      </c>
+    </row>
+    <row r="187" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A187" s="39" t="s">
+        <v>394</v>
+      </c>
+      <c r="B187" s="40"/>
+      <c r="C187" s="41" t="s">
+        <v>395</v>
+      </c>
+      <c r="D187" s="41"/>
+      <c r="E187" s="40"/>
+      <c r="F187" s="40"/>
+      <c r="G187" s="40"/>
+      <c r="H187" s="41"/>
+      <c r="I187" s="41"/>
+      <c r="J187" s="40" t="str">
+        <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G187)</f>
+        <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#</v>
+      </c>
+      <c r="K187" s="40" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="188" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A188" s="42"/>
+      <c r="B188" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="C188" s="10" t="s">
+        <v>141</v>
+      </c>
+      <c r="G188" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="J188" s="1" t="str">
+        <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G188)</f>
+        <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#hasIdentifier</v>
+      </c>
+    </row>
+    <row r="189" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A189" s="42"/>
+      <c r="B189" s="11"/>
+      <c r="J189" s="1" t="str">
+        <f aca="false">_xlfn.CONCAT("https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#", G189)</f>
         <v>https://github.com/gryvity/miafpe/tree/master/ontology/miappexsosa.owl#</v>
       </c>
     </row>
@@ -5545,6 +5829,168 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData/>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData/>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData/>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData/>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData/>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData/>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData/>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData/>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData/>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -5584,61 +6030,61 @@
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="11" style="1" width="11.53"/>
   </cols>
   <sheetData>
-    <row r="1" s="25" customFormat="true" ht="36.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="25" t="s">
+    <row r="1" s="24" customFormat="true" ht="36.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="B1" s="25" t="s">
+      <c r="B1" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="C1" s="25" t="s">
+      <c r="C1" s="24" t="s">
         <v>29</v>
       </c>
-      <c r="D1" s="25" t="s">
+      <c r="D1" s="24" t="s">
         <v>35</v>
       </c>
-      <c r="E1" s="25" t="s">
+      <c r="E1" s="24" t="s">
         <v>40</v>
       </c>
-      <c r="F1" s="25" t="s">
+      <c r="F1" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="G1" s="25" t="s">
+      <c r="G1" s="24" t="s">
         <v>49</v>
       </c>
-      <c r="H1" s="25" t="s">
+      <c r="H1" s="24" t="s">
         <v>53</v>
       </c>
-      <c r="I1" s="42" t="s">
+      <c r="I1" s="43" t="s">
         <v>57</v>
       </c>
-      <c r="J1" s="25" t="s">
-        <v>354</v>
-      </c>
-    </row>
-    <row r="2" s="36" customFormat="true" ht="124.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="36" t="s">
-        <v>355</v>
-      </c>
-      <c r="B2" s="36" t="s">
-        <v>356</v>
-      </c>
-      <c r="C2" s="36" t="s">
-        <v>357</v>
-      </c>
-      <c r="D2" s="43" t="n">
+      <c r="J1" s="24" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="2" s="35" customFormat="true" ht="124.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="35" t="s">
+        <v>397</v>
+      </c>
+      <c r="B2" s="35" t="s">
+        <v>398</v>
+      </c>
+      <c r="C2" s="35" t="s">
+        <v>399</v>
+      </c>
+      <c r="D2" s="44" t="n">
         <v>45644</v>
       </c>
-      <c r="E2" s="43" t="n">
+      <c r="E2" s="44" t="n">
         <v>45644</v>
       </c>
-      <c r="F2" s="36" t="s">
-        <v>358</v>
-      </c>
-      <c r="G2" s="36" t="n">
+      <c r="F2" s="35" t="s">
+        <v>400</v>
+      </c>
+      <c r="G2" s="35" t="n">
         <v>3.2</v>
       </c>
-      <c r="H2" s="36" t="n">
+      <c r="H2" s="35" t="n">
         <v>0.1</v>
       </c>
     </row>
@@ -5662,42 +6108,42 @@
   <dimension ref="A1:I1"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="31" width="20.75"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="31" width="14.03"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="31" width="19.24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="31" width="14.94"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="31" width="13.1"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="31" width="17.04"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="31" width="18.08"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="31" width="21.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="30" width="20.75"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="30" width="14.03"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="30" width="19.24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="30" width="14.94"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="30" width="13.1"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="30" width="17.04"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="30" width="18.08"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="30" width="21.79"/>
   </cols>
   <sheetData>
-    <row r="1" s="42" customFormat="true" ht="36.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="42" t="s">
+    <row r="1" s="43" customFormat="true" ht="36.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="43" t="s">
         <v>73</v>
       </c>
-      <c r="B1" s="42" t="s">
+      <c r="B1" s="43" t="s">
         <v>77</v>
       </c>
-      <c r="C1" s="42" t="s">
+      <c r="C1" s="43" t="s">
         <v>80</v>
       </c>
-      <c r="D1" s="42" t="s">
+      <c r="D1" s="43" t="s">
         <v>83</v>
       </c>
-      <c r="E1" s="42" t="s">
+      <c r="E1" s="43" t="s">
         <v>86</v>
       </c>
-      <c r="F1" s="42" t="s">
+      <c r="F1" s="43" t="s">
         <v>89</v>
       </c>
-      <c r="G1" s="42" t="s">
+      <c r="G1" s="43" t="s">
         <v>93</v>
       </c>
-      <c r="H1" s="42" t="s">
+      <c r="H1" s="43" t="s">
         <v>96</v>
       </c>
-      <c r="I1" s="42" t="s">
+      <c r="I1" s="43" t="s">
         <v>100</v>
       </c>
     </row>
@@ -5720,34 +6166,34 @@
   <dimension ref="A1:F1"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="31" width="24.56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="31" width="14.03"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="31" width="19.24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="31" width="14.94"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="31" width="13.1"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="31" width="17.04"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="31" width="18.08"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="31" width="21.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="30" width="24.56"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="30" width="14.03"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="30" width="19.24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="30" width="14.94"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="30" width="13.1"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="30" width="17.04"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="30" width="18.08"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="30" width="21.79"/>
   </cols>
   <sheetData>
-    <row r="1" s="42" customFormat="true" ht="36.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="42" t="s">
-        <v>329</v>
-      </c>
-      <c r="B1" s="42" t="s">
-        <v>330</v>
-      </c>
-      <c r="C1" s="42" t="s">
-        <v>332</v>
-      </c>
-      <c r="D1" s="42" t="s">
-        <v>335</v>
-      </c>
-      <c r="E1" s="42" t="s">
-        <v>338</v>
-      </c>
-      <c r="F1" s="42" t="s">
-        <v>341</v>
+    <row r="1" s="43" customFormat="true" ht="36.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="43" t="s">
+        <v>371</v>
+      </c>
+      <c r="B1" s="43" t="s">
+        <v>372</v>
+      </c>
+      <c r="C1" s="43" t="s">
+        <v>374</v>
+      </c>
+      <c r="D1" s="43" t="s">
+        <v>377</v>
+      </c>
+      <c r="E1" s="43" t="s">
+        <v>380</v>
+      </c>
+      <c r="F1" s="43" t="s">
+        <v>383</v>
       </c>
     </row>
   </sheetData>
@@ -5769,33 +6215,33 @@
   <dimension ref="A1:F1"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="31" width="20.75"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="31" width="14.03"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="31" width="19.24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="31" width="20.24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="31" width="13.1"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="31" width="17.04"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="31" width="18.08"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="31" width="21.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="30" width="20.75"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="30" width="14.03"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="30" width="19.24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="30" width="20.24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="30" width="13.1"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="30" width="17.04"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="30" width="18.08"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="30" width="21.79"/>
   </cols>
   <sheetData>
-    <row r="1" s="42" customFormat="true" ht="36.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="44" t="s">
+    <row r="1" s="43" customFormat="true" ht="36.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="45" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="44" t="s">
+      <c r="B1" s="45" t="s">
         <v>176</v>
       </c>
-      <c r="C1" s="44" t="s">
+      <c r="C1" s="45" t="s">
         <v>180</v>
       </c>
-      <c r="D1" s="44" t="s">
+      <c r="D1" s="45" t="s">
         <v>182</v>
       </c>
-      <c r="E1" s="44" t="s">
+      <c r="E1" s="45" t="s">
         <v>184</v>
       </c>
-      <c r="F1" s="44" t="s">
+      <c r="F1" s="45" t="s">
         <v>187</v>
       </c>
     </row>
@@ -5818,45 +6264,45 @@
   <dimension ref="A1:J1"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="31" width="20.75"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="31" width="14.03"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="31" width="19.24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="31" width="14.94"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="31" width="13.1"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="31" width="17.04"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="31" width="18.08"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="31" width="21.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="30" width="20.75"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="30" width="14.03"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="30" width="19.24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="30" width="14.94"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="30" width="13.1"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="30" width="17.04"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="30" width="18.08"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="30" width="21.79"/>
   </cols>
   <sheetData>
-    <row r="1" s="42" customFormat="true" ht="36.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="25" t="s">
+    <row r="1" s="43" customFormat="true" ht="36.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="24" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="25" t="s">
+      <c r="B1" s="24" t="s">
         <v>105</v>
       </c>
-      <c r="C1" s="25" t="s">
+      <c r="C1" s="24" t="s">
         <v>107</v>
       </c>
-      <c r="D1" s="25" t="s">
+      <c r="D1" s="24" t="s">
         <v>111</v>
       </c>
-      <c r="E1" s="25" t="s">
+      <c r="E1" s="24" t="s">
         <v>114</v>
       </c>
-      <c r="F1" s="25" t="s">
+      <c r="F1" s="24" t="s">
         <v>119</v>
       </c>
-      <c r="G1" s="25" t="s">
+      <c r="G1" s="24" t="s">
         <v>123</v>
       </c>
-      <c r="H1" s="25" t="s">
+      <c r="H1" s="24" t="s">
         <v>132</v>
       </c>
-      <c r="I1" s="25" t="s">
+      <c r="I1" s="24" t="s">
         <v>135</v>
       </c>
-      <c r="J1" s="25" t="s">
+      <c r="J1" s="24" t="s">
         <v>138</v>
       </c>
     </row>
@@ -5879,51 +6325,51 @@
   <dimension ref="A1:L1"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="31" width="20.75"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="31" width="14.03"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="31" width="19.24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="31" width="14.94"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="31" width="13.1"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="31" width="17.04"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="31" width="18.08"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="31" width="21.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="30" width="20.75"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="30" width="14.03"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="30" width="19.24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="30" width="14.94"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="30" width="13.1"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="30" width="17.04"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="30" width="18.08"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="30" width="21.79"/>
   </cols>
   <sheetData>
-    <row r="1" s="42" customFormat="true" ht="36.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="44" t="s">
+    <row r="1" s="43" customFormat="true" ht="36.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="45" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="44" t="s">
+      <c r="B1" s="45" t="s">
         <v>142</v>
       </c>
-      <c r="C1" s="44" t="s">
+      <c r="C1" s="45" t="s">
         <v>144</v>
       </c>
-      <c r="D1" s="44" t="s">
+      <c r="D1" s="45" t="s">
         <v>107</v>
       </c>
-      <c r="E1" s="44" t="s">
+      <c r="E1" s="45" t="s">
         <v>111</v>
       </c>
-      <c r="F1" s="44" t="s">
+      <c r="F1" s="45" t="s">
         <v>147</v>
       </c>
-      <c r="G1" s="44" t="s">
+      <c r="G1" s="45" t="s">
         <v>150</v>
       </c>
-      <c r="H1" s="44" t="s">
+      <c r="H1" s="45" t="s">
         <v>152</v>
       </c>
-      <c r="I1" s="44" t="s">
+      <c r="I1" s="45" t="s">
         <v>154</v>
       </c>
-      <c r="J1" s="44" t="s">
+      <c r="J1" s="45" t="s">
         <v>156</v>
       </c>
-      <c r="K1" s="44" t="s">
+      <c r="K1" s="45" t="s">
         <v>158</v>
       </c>
-      <c r="L1" s="44" t="s">
+      <c r="L1" s="45" t="s">
         <v>160</v>
       </c>
     </row>
@@ -5946,30 +6392,30 @@
   <dimension ref="A1:E1"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="31" width="20.75"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="31" width="14.03"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="31" width="19.24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="31" width="14.94"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="31" width="13.1"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="31" width="17.04"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="31" width="18.08"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="31" width="21.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="30" width="20.75"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="30" width="14.03"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="30" width="19.24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="30" width="14.94"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="30" width="13.1"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="30" width="17.04"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="30" width="18.08"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="30" width="21.79"/>
   </cols>
   <sheetData>
-    <row r="1" s="42" customFormat="true" ht="36.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="44" t="s">
+    <row r="1" s="43" customFormat="true" ht="36.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="45" t="s">
         <v>163</v>
       </c>
-      <c r="B1" s="44" t="s">
+      <c r="B1" s="45" t="s">
         <v>164</v>
       </c>
-      <c r="C1" s="44" t="s">
+      <c r="C1" s="45" t="s">
         <v>166</v>
       </c>
-      <c r="D1" s="44" t="s">
+      <c r="D1" s="45" t="s">
         <v>168</v>
       </c>
-      <c r="E1" s="44" t="s">
+      <c r="E1" s="45" t="s">
         <v>171</v>
       </c>
     </row>

</xml_diff>